<commit_message>
fiscal: phase 1 source cards + audit refresh.
- editorial/source_cards/_pending/fiscal/ — four source cards for the
  new /fiscal/ section plates (plate-2 debt-service share, plate-3 PBO
  vs DoF SEU, plate-4 four-province net debt-to-GDP, plate-5 CAPB).
  Awaiting Jay's review per the plan's Phase 1 user-review gate before
  Phase 2 dispatches.
- editorial/source_cards/audit/ — built audit tables regenerated.
- bylines/commentaries/ — xlsx working-file touches from the retail
  commentary cycle.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bylines/commentaries/Sibley Creek Inflation Chart Template.xlsx
+++ b/bylines/commentaries/Sibley Creek Inflation Chart Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayzh\projects\macro-research-department\bylines\commentaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75BD03C8-12F0-48F7-9411-07061C7BB475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FEFB0EB-3346-4637-8538-51B684F50728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -129,8 +129,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="mmm\ yyyy"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="mmm\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -186,12 +186,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2020,8 +2020,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5009216" y="129887"/>
-          <a:ext cx="4830932" cy="2784079"/>
+          <a:off x="4988611" y="129887"/>
+          <a:ext cx="4858655" cy="2805058"/>
           <a:chOff x="4991881" y="129887"/>
           <a:chExt cx="4855749" cy="2795757"/>
         </a:xfrm>
@@ -2572,7 +2572,7 @@
         <v>0.33579583613163599</v>
       </c>
       <c r="D14" s="4" t="str">
-        <f>IFERROR((B14/B2-1)*100,"")</f>
+        <f t="shared" ref="D14:D45" si="2">IFERROR((B14/B2-1)*100,"")</f>
         <v/>
       </c>
       <c r="E14" s="4">
@@ -2592,7 +2592,7 @@
         <v>1.1378848728246238</v>
       </c>
       <c r="D15" s="4">
-        <f>IFERROR((B15/B3-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>7.6977904490377558</v>
       </c>
       <c r="E15" s="4">
@@ -2612,7 +2612,7 @@
         <v>0.72799470549305134</v>
       </c>
       <c r="D16" s="4">
-        <f>IFERROR((B16/B4-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>8.1734186211798168</v>
       </c>
       <c r="E16" s="4">
@@ -2632,7 +2632,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="4">
-        <f>IFERROR((B17/B5-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>7.6379066478076352</v>
       </c>
       <c r="E17" s="4">
@@ -2652,7 +2652,7 @@
         <v>-6.5703022339025363E-2</v>
       </c>
       <c r="D18" s="4">
-        <f>IFERROR((B18/B6-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>6.8868587491215605</v>
       </c>
       <c r="E18" s="4">
@@ -2672,7 +2672,7 @@
         <v>0.46022353714663122</v>
       </c>
       <c r="D19" s="4">
-        <f>IFERROR((B19/B7-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>6.7784765897973553</v>
       </c>
       <c r="E19" s="4">
@@ -2692,7 +2692,7 @@
         <v>0.58900523560208029</v>
       </c>
       <c r="D20" s="4">
-        <f>IFERROR((B20/B8-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>6.8102849200833759</v>
       </c>
       <c r="E20" s="4">
@@ -2712,7 +2712,7 @@
         <v>0.39037085230970714</v>
       </c>
       <c r="D21" s="4">
-        <f>IFERROR((B21/B9-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>6.78200692041524</v>
       </c>
       <c r="E21" s="4">
@@ -2732,7 +2732,7 @@
         <v>-6.4808813998717962E-2</v>
       </c>
       <c r="D22" s="4">
-        <f>IFERROR((B22/B10-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>6.198347107438007</v>
       </c>
       <c r="E22" s="4">
@@ -2752,7 +2752,7 @@
         <v>0.45395590142673914</v>
       </c>
       <c r="D23" s="4">
-        <f>IFERROR((B23/B11-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>5.8783321941216604</v>
       </c>
       <c r="E23" s="4">
@@ -2772,7 +2772,7 @@
         <v>0.12911555842478606</v>
       </c>
       <c r="D24" s="4">
-        <f>IFERROR((B24/B12-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>5.2953156822810543</v>
       </c>
       <c r="E24" s="4">
@@ -2792,7 +2792,7 @@
         <v>0.12894906511928816</v>
       </c>
       <c r="D25" s="4">
-        <f>IFERROR((B25/B13-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>4.2981867024848963</v>
       </c>
       <c r="E25" s="4">
@@ -2812,7 +2812,7 @@
         <v>0.51513200257564673</v>
       </c>
       <c r="D26" s="4">
-        <f>IFERROR((B26/B14-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>4.4846050870147147</v>
       </c>
       <c r="E26" s="4">
@@ -2832,7 +2832,7 @@
         <v>6.4061499039080871E-2</v>
       </c>
       <c r="D27" s="4">
-        <f>IFERROR((B27/B15-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.3752481800132239</v>
       </c>
       <c r="E27" s="4">
@@ -2852,7 +2852,7 @@
         <v>0.25608194622279701</v>
       </c>
       <c r="D28" s="4">
-        <f>IFERROR((B28/B16-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>2.890932982917227</v>
       </c>
       <c r="E28" s="4">
@@ -2872,7 +2872,7 @@
         <v>0.38314176245211051</v>
       </c>
       <c r="D29" s="4">
-        <f>IFERROR((B29/B17-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.2851511169513792</v>
       </c>
       <c r="E29" s="4">
@@ -2892,7 +2892,7 @@
         <v>0.69974554707381564</v>
       </c>
       <c r="D30" s="4">
-        <f>IFERROR((B30/B18-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>4.0762656147271592</v>
       </c>
       <c r="E30" s="4">
@@ -2912,7 +2912,7 @@
         <v>0.18951358180667732</v>
       </c>
       <c r="D31" s="4">
-        <f>IFERROR((B31/B19-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.7958115183245988</v>
       </c>
       <c r="E31" s="4">
@@ -2932,7 +2932,7 @@
         <v>-6.3051702395966469E-2</v>
       </c>
       <c r="D32" s="4">
-        <f>IFERROR((B32/B20-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.1229668184775683</v>
       </c>
       <c r="E32" s="4">
@@ -2952,7 +2952,7 @@
         <v>0.3154574132492094</v>
       </c>
       <c r="D33" s="4">
-        <f>IFERROR((B33/B21-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.046014257939067</v>
       </c>
       <c r="E33" s="4">
@@ -2972,7 +2972,7 @@
         <v>0.2515723270440251</v>
       </c>
       <c r="D34" s="4">
-        <f>IFERROR((B34/B22-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>3.3722438391699194</v>
       </c>
       <c r="E34" s="4">
@@ -2988,11 +2988,11 @@
         <v>159.4</v>
       </c>
       <c r="C35" s="4">
-        <f t="shared" ref="C35:C66" si="2">IFERROR((B35/B34-1)*100,"")</f>
+        <f t="shared" ref="C35:C66" si="3">IFERROR((B35/B34-1)*100,"")</f>
         <v>0</v>
       </c>
       <c r="D35" s="4">
-        <f>IFERROR((B35/B23-1)*100,"")</f>
+        <f t="shared" si="2"/>
         <v>2.9051000645577751</v>
       </c>
       <c r="E35" s="4">
@@ -3008,11 +3008,11 @@
         <v>159.4</v>
       </c>
       <c r="C36" s="4">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D36" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="D36" s="4">
-        <f>IFERROR((B36/B24-1)*100,"")</f>
         <v>2.7724049000644735</v>
       </c>
       <c r="E36" s="4">
@@ -3028,15 +3028,15 @@
         <v>159.80000000000001</v>
       </c>
       <c r="C37" s="4">
+        <f t="shared" si="3"/>
+        <v>0.25094102885823144</v>
+      </c>
+      <c r="D37" s="4">
         <f t="shared" si="2"/>
-        <v>0.25094102885823144</v>
-      </c>
-      <c r="D37" s="4">
-        <f>IFERROR((B37/B25-1)*100,"")</f>
         <v>2.8976175144880933</v>
       </c>
       <c r="E37" s="4">
-        <f t="shared" ref="E37:E68" si="3">IFERROR(((B37/B34)^4-1)*100,"")</f>
+        <f t="shared" ref="E37:E68" si="4">IFERROR(((B37/B34)^4-1)*100,"")</f>
         <v>1.0075487242393155</v>
       </c>
     </row>
@@ -3048,15 +3048,15 @@
         <v>160.30000000000001</v>
       </c>
       <c r="C38" s="4">
+        <f t="shared" si="3"/>
+        <v>0.31289111389236623</v>
+      </c>
+      <c r="D38" s="4">
         <f t="shared" si="2"/>
-        <v>0.31289111389236623</v>
-      </c>
-      <c r="D38" s="4">
-        <f>IFERROR((B38/B26-1)*100,"")</f>
         <v>2.6905829596412634</v>
       </c>
       <c r="E38" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.2776689224460966</v>
       </c>
     </row>
@@ -3068,15 +3068,15 @@
         <v>160.69999999999999</v>
       </c>
       <c r="C39" s="4">
+        <f t="shared" si="3"/>
+        <v>0.24953212726137597</v>
+      </c>
+      <c r="D39" s="4">
         <f t="shared" si="2"/>
-        <v>0.24953212726137597</v>
-      </c>
-      <c r="D39" s="4">
-        <f>IFERROR((B39/B27-1)*100,"")</f>
         <v>2.8809218950063942</v>
       </c>
       <c r="E39" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.3023589249833618</v>
       </c>
     </row>
@@ -3088,15 +3088,15 @@
         <v>160.80000000000001</v>
       </c>
       <c r="C40" s="4">
+        <f t="shared" si="3"/>
+        <v>6.2227753578114609E-2</v>
+      </c>
+      <c r="D40" s="4">
         <f t="shared" si="2"/>
-        <v>6.2227753578114609E-2</v>
-      </c>
-      <c r="D40" s="4">
-        <f>IFERROR((B40/B28-1)*100,"")</f>
         <v>2.6819923371647514</v>
       </c>
       <c r="E40" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.52672329166721</v>
       </c>
     </row>
@@ -3108,15 +3108,15 @@
         <v>161.19999999999999</v>
       </c>
       <c r="C41" s="4">
+        <f t="shared" si="3"/>
+        <v>0.24875621890545485</v>
+      </c>
+      <c r="D41" s="4">
         <f t="shared" si="2"/>
-        <v>0.24875621890545485</v>
-      </c>
-      <c r="D41" s="4">
-        <f>IFERROR((B41/B29-1)*100,"")</f>
         <v>2.5445292620865034</v>
       </c>
       <c r="E41" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.2647734204898073</v>
       </c>
     </row>
@@ -3128,15 +3128,15 @@
         <v>161.30000000000001</v>
       </c>
       <c r="C42" s="4">
+        <f t="shared" si="3"/>
+        <v>6.2034739454097654E-2</v>
+      </c>
+      <c r="D42" s="4">
         <f t="shared" si="2"/>
-        <v>6.2034739454097654E-2</v>
-      </c>
-      <c r="D42" s="4">
-        <f>IFERROR((B42/B30-1)*100,"")</f>
         <v>1.8951358180669509</v>
       </c>
       <c r="E42" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.5018510781681593</v>
       </c>
     </row>
@@ -3148,15 +3148,15 @@
         <v>161.19999999999999</v>
       </c>
       <c r="C43" s="4">
+        <f t="shared" si="3"/>
+        <v>-6.1996280223197697E-2</v>
+      </c>
+      <c r="D43" s="4">
         <f t="shared" si="2"/>
-        <v>-6.1996280223197697E-2</v>
-      </c>
-      <c r="D43" s="4">
-        <f>IFERROR((B43/B31-1)*100,"")</f>
         <v>1.6393442622950838</v>
       </c>
       <c r="E43" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.99874381601730011</v>
       </c>
     </row>
@@ -3168,15 +3168,15 @@
         <v>161.69999999999999</v>
       </c>
       <c r="C44" s="4">
+        <f t="shared" si="3"/>
+        <v>0.31017369727046606</v>
+      </c>
+      <c r="D44" s="4">
         <f t="shared" si="2"/>
-        <v>0.31017369727046606</v>
-      </c>
-      <c r="D44" s="4">
-        <f>IFERROR((B44/B32-1)*100,"")</f>
         <v>2.018927444794949</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.2464791981284806</v>
       </c>
     </row>
@@ -3188,15 +3188,15 @@
         <v>162</v>
       </c>
       <c r="C45" s="4">
+        <f t="shared" si="3"/>
+        <v>0.18552875695734272</v>
+      </c>
+      <c r="D45" s="4">
         <f t="shared" si="2"/>
-        <v>0.18552875695734272</v>
-      </c>
-      <c r="D45" s="4">
-        <f>IFERROR((B45/B33-1)*100,"")</f>
         <v>1.8867924528301883</v>
       </c>
       <c r="E45" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.7472285783940888</v>
       </c>
     </row>
@@ -3208,15 +3208,15 @@
         <v>162.30000000000001</v>
       </c>
       <c r="C46" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.18518518518519933</v>
       </c>
       <c r="D46" s="4">
-        <f>IFERROR((B46/B34-1)*100,"")</f>
+        <f t="shared" ref="D46:D77" si="5">IFERROR((B46/B34-1)*100,"")</f>
         <v>1.8193224592220947</v>
       </c>
       <c r="E46" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.7575945746479036</v>
       </c>
     </row>
@@ -3228,15 +3228,15 @@
         <v>162.5</v>
       </c>
       <c r="C47" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.12322858903264233</v>
       </c>
       <c r="D47" s="4">
-        <f>IFERROR((B47/B35-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.9447929736511993</v>
       </c>
       <c r="E47" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.993708166038699</v>
       </c>
     </row>
@@ -3248,15 +3248,15 @@
         <v>163.5</v>
       </c>
       <c r="C48" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.61538461538461764</v>
       </c>
       <c r="D48" s="4">
-        <f>IFERROR((B48/B36-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.5721455457967446</v>
       </c>
       <c r="E48" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.7554623008480892</v>
       </c>
     </row>
@@ -3268,15 +3268,15 @@
         <v>163.5</v>
       </c>
       <c r="C49" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="D49" s="4">
-        <f>IFERROR((B49/B37-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.3153942428034924</v>
       </c>
       <c r="E49" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.9904483285400074</v>
       </c>
     </row>
@@ -3288,15 +3288,15 @@
         <v>163.1</v>
       </c>
       <c r="C50" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.24464831804281717</v>
       </c>
       <c r="D50" s="4">
-        <f>IFERROR((B50/B38-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.7467248908296762</v>
       </c>
       <c r="E50" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.4851231122594344</v>
       </c>
     </row>
@@ -3308,15 +3308,15 @@
         <v>163.5</v>
       </c>
       <c r="C51" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.24524831391785629</v>
       </c>
       <c r="D51" s="4">
-        <f>IFERROR((B51/B39-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.7423771001866983</v>
       </c>
       <c r="E51" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -3328,15 +3328,15 @@
         <v>163.9</v>
       </c>
       <c r="C52" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.24464831804280607</v>
       </c>
       <c r="D52" s="4">
-        <f>IFERROR((B52/B40-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.9278606965174028</v>
       </c>
       <c r="E52" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.9821903008795374</v>
       </c>
     </row>
@@ -3348,15 +3348,15 @@
         <v>164</v>
       </c>
       <c r="C53" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.1012812690663942E-2</v>
       </c>
       <c r="D53" s="4">
-        <f>IFERROR((B53/B41-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.7369727047146455</v>
       </c>
       <c r="E53" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.2255716976002704</v>
       </c>
     </row>
@@ -3368,15 +3368,15 @@
         <v>164.3</v>
       </c>
       <c r="C54" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.18292682926830395</v>
       </c>
       <c r="D54" s="4">
-        <f>IFERROR((B54/B42-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.8598884066955979</v>
       </c>
       <c r="E54" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.9715981307828701</v>
       </c>
     </row>
@@ -3388,15 +3388,15 @@
         <v>165</v>
       </c>
       <c r="C55" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.42604990870358517</v>
       </c>
       <c r="D55" s="4">
-        <f>IFERROR((B55/B43-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.3573200992555998</v>
       </c>
       <c r="E55" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.7117106917732947</v>
       </c>
     </row>
@@ -3408,15 +3408,15 @@
         <v>165.2</v>
       </c>
       <c r="C56" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.12121212121212199</v>
       </c>
       <c r="D56" s="4">
-        <f>IFERROR((B56/B44-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.1645021645021689</v>
       </c>
       <c r="E56" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.9591099919632269</v>
       </c>
     </row>
@@ -3428,15 +3428,15 @@
         <v>165.6</v>
       </c>
       <c r="C57" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.2421307506053294</v>
       </c>
       <c r="D57" s="4">
-        <f>IFERROR((B57/B45-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.2222222222222143</v>
       </c>
       <c r="E57" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.2027039344914021</v>
       </c>
     </row>
@@ -3448,15 +3448,15 @@
         <v>166.1</v>
       </c>
       <c r="C58" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.30193236714974869</v>
       </c>
       <c r="D58" s="4">
-        <f>IFERROR((B58/B46-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.3413431916204486</v>
       </c>
       <c r="E58" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.6934520493826941</v>
       </c>
     </row>
@@ -3468,15 +3468,15 @@
         <v>166.2</v>
       </c>
       <c r="C59" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.0204695966281641E-2</v>
       </c>
       <c r="D59" s="4">
-        <f>IFERROR((B59/B47-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.2769230769230653</v>
       </c>
       <c r="E59" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.4433815996646402</v>
       </c>
     </row>
@@ -3488,15 +3488,15 @@
         <v>166.5</v>
       </c>
       <c r="C60" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.18050541516245744</v>
       </c>
       <c r="D60" s="4">
-        <f>IFERROR((B60/B48-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>1.8348623853210899</v>
       </c>
       <c r="E60" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.1916994584927796</v>
       </c>
     </row>
@@ -3508,15 +3508,15 @@
         <v>167.3</v>
       </c>
       <c r="C61" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.48048048048048297</v>
       </c>
       <c r="D61" s="4">
-        <f>IFERROR((B61/B49-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.3241590214067243</v>
       </c>
       <c r="E61" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.9212931020702326</v>
       </c>
     </row>
@@ -3528,841 +3528,841 @@
         <v>167.8</v>
       </c>
       <c r="C62" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.29886431560071092</v>
       </c>
       <c r="D62" s="4">
-        <f>IFERROR((B62/B50-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>2.8816676885346615</v>
       </c>
       <c r="E62" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.9067468959312013</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C63" s="4">
-        <f t="shared" si="2"/>
-        <v>-100</v>
-      </c>
-      <c r="D63" s="4">
-        <f>IFERROR((B63/B51-1)*100,"")</f>
-        <v>-100</v>
-      </c>
-      <c r="E63" s="4">
         <f t="shared" si="3"/>
         <v>-100</v>
       </c>
+      <c r="D63" s="4">
+        <f t="shared" si="5"/>
+        <v>-100</v>
+      </c>
+      <c r="E63" s="4">
+        <f t="shared" si="4"/>
+        <v>-100</v>
+      </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C64" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="D64" s="4">
-        <f>IFERROR((B64/B52-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E64" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-100</v>
       </c>
     </row>
     <row r="65" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C65" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="D65" s="4">
-        <f>IFERROR((B65/B53-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E65" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-100</v>
       </c>
     </row>
     <row r="66" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C66" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="D66" s="4">
-        <f>IFERROR((B66/B54-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E66" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="67" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C67" s="4" t="str">
-        <f t="shared" ref="C67:C98" si="4">IFERROR((B67/B66-1)*100,"")</f>
+        <f t="shared" ref="C67:C98" si="6">IFERROR((B67/B66-1)*100,"")</f>
         <v/>
       </c>
       <c r="D67" s="4">
-        <f>IFERROR((B67/B55-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E67" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="68" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C68" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="D68" s="4">
+        <f t="shared" si="5"/>
+        <v>-100</v>
+      </c>
+      <c r="E68" s="4" t="str">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="D68" s="4">
-        <f>IFERROR((B68/B56-1)*100,"")</f>
-        <v>-100</v>
-      </c>
-      <c r="E68" s="4" t="str">
-        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="69" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C69" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D69" s="4">
-        <f>IFERROR((B69/B57-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E69" s="4" t="str">
-        <f t="shared" ref="E69:E100" si="5">IFERROR(((B69/B66)^4-1)*100,"")</f>
+        <f t="shared" ref="E69:E100" si="7">IFERROR(((B69/B66)^4-1)*100,"")</f>
         <v/>
       </c>
     </row>
     <row r="70" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C70" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D70" s="4">
-        <f>IFERROR((B70/B58-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E70" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="71" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C71" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D71" s="4">
-        <f>IFERROR((B71/B59-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E71" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="72" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C72" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D72" s="4">
-        <f>IFERROR((B72/B60-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E72" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="73" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C73" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D73" s="4">
-        <f>IFERROR((B73/B61-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E73" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="74" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C74" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D74" s="4">
-        <f>IFERROR((B74/B62-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v>-100</v>
       </c>
       <c r="E74" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="75" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C75" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D75" s="4" t="str">
-        <f>IFERROR((B75/B63-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="E75" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="76" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C76" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D76" s="4" t="str">
-        <f>IFERROR((B76/B64-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="E76" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="77" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C77" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D77" s="4" t="str">
-        <f>IFERROR((B77/B65-1)*100,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="E77" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="78" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C78" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D78" s="4" t="str">
-        <f>IFERROR((B78/B66-1)*100,"")</f>
+        <f t="shared" ref="D78:D109" si="8">IFERROR((B78/B66-1)*100,"")</f>
         <v/>
       </c>
       <c r="E78" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="79" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C79" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D79" s="4" t="str">
-        <f>IFERROR((B79/B67-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E79" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="80" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C80" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D80" s="4" t="str">
-        <f>IFERROR((B80/B68-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E80" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="81" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C81" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D81" s="4" t="str">
-        <f>IFERROR((B81/B69-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E81" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="82" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C82" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D82" s="4" t="str">
-        <f>IFERROR((B82/B70-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E82" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="83" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C83" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D83" s="4" t="str">
-        <f>IFERROR((B83/B71-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E83" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="84" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C84" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D84" s="4" t="str">
-        <f>IFERROR((B84/B72-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E84" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="85" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C85" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D85" s="4" t="str">
-        <f>IFERROR((B85/B73-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E85" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="86" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C86" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D86" s="4" t="str">
-        <f>IFERROR((B86/B74-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E86" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="87" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C87" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D87" s="4" t="str">
-        <f>IFERROR((B87/B75-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E87" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="88" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C88" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D88" s="4" t="str">
-        <f>IFERROR((B88/B76-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E88" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="89" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C89" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D89" s="4" t="str">
-        <f>IFERROR((B89/B77-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E89" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="90" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C90" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D90" s="4" t="str">
-        <f>IFERROR((B90/B78-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E90" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="91" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C91" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D91" s="4" t="str">
-        <f>IFERROR((B91/B79-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E91" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="92" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C92" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D92" s="4" t="str">
-        <f>IFERROR((B92/B80-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E92" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="93" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C93" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D93" s="4" t="str">
-        <f>IFERROR((B93/B81-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E93" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="94" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C94" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D94" s="4" t="str">
-        <f>IFERROR((B94/B82-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E94" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="95" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C95" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D95" s="4" t="str">
-        <f>IFERROR((B95/B83-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E95" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="96" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C96" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D96" s="4" t="str">
-        <f>IFERROR((B96/B84-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E96" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="97" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C97" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D97" s="4" t="str">
-        <f>IFERROR((B97/B85-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E97" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="98" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C98" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="D98" s="4" t="str">
-        <f>IFERROR((B98/B86-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E98" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="99" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C99" s="4" t="str">
-        <f t="shared" ref="C99:C121" si="6">IFERROR((B99/B98-1)*100,"")</f>
+        <f t="shared" ref="C99:C121" si="9">IFERROR((B99/B98-1)*100,"")</f>
         <v/>
       </c>
       <c r="D99" s="4" t="str">
-        <f>IFERROR((B99/B87-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E99" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="100" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C100" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D100" s="4" t="str">
-        <f>IFERROR((B100/B88-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E100" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="101" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C101" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D101" s="4" t="str">
-        <f>IFERROR((B101/B89-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E101" s="4" t="str">
-        <f t="shared" ref="E101:E132" si="7">IFERROR(((B101/B98)^4-1)*100,"")</f>
+        <f t="shared" ref="E101:E121" si="10">IFERROR(((B101/B98)^4-1)*100,"")</f>
         <v/>
       </c>
     </row>
     <row r="102" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C102" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D102" s="4" t="str">
-        <f>IFERROR((B102/B90-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E102" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="103" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C103" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D103" s="4" t="str">
-        <f>IFERROR((B103/B91-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E103" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="104" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C104" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D104" s="4" t="str">
-        <f>IFERROR((B104/B92-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E104" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="105" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C105" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D105" s="4" t="str">
-        <f>IFERROR((B105/B93-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E105" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="106" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C106" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D106" s="4" t="str">
-        <f>IFERROR((B106/B94-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E106" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="107" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C107" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D107" s="4" t="str">
-        <f>IFERROR((B107/B95-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E107" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="108" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C108" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D108" s="4" t="str">
-        <f>IFERROR((B108/B96-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E108" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="109" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C109" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D109" s="4" t="str">
-        <f>IFERROR((B109/B97-1)*100,"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="E109" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="110" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C110" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D110" s="4" t="str">
-        <f>IFERROR((B110/B98-1)*100,"")</f>
+        <f t="shared" ref="D110:D141" si="11">IFERROR((B110/B98-1)*100,"")</f>
         <v/>
       </c>
       <c r="E110" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="111" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C111" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D111" s="4" t="str">
-        <f>IFERROR((B111/B99-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E111" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="112" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C112" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D112" s="4" t="str">
-        <f>IFERROR((B112/B100-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E112" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C113" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D113" s="4" t="str">
-        <f>IFERROR((B113/B101-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E113" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C114" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D114" s="4" t="str">
-        <f>IFERROR((B114/B102-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E114" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C115" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D115" s="4" t="str">
-        <f>IFERROR((B115/B103-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E115" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C116" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D116" s="4" t="str">
-        <f>IFERROR((B116/B104-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E116" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C117" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D117" s="4" t="str">
-        <f>IFERROR((B117/B105-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E117" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C118" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D118" s="4" t="str">
-        <f>IFERROR((B118/B106-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E118" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C119" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D119" s="4" t="str">
-        <f>IFERROR((B119/B107-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E119" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C120" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D120" s="4" t="str">
-        <f>IFERROR((B120/B108-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E120" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C121" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="D121" s="4" t="str">
-        <f>IFERROR((B121/B109-1)*100,"")</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="E121" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>

</xml_diff>